<commit_message>
calcula inercia, deflexion teorica y diferencia relativa en analisis_viga.xlsx
</commit_message>
<xml_diff>
--- a/analysis/analisis_viga.xlsx
+++ b/analysis/analisis_viga.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\galej\Desktop\EVALUACION 1\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{E83AB9F2-077B-42D1-89AE-3AC5D308DB7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B16B76B5-5DF2-46A3-9E7B-9860B0FA41C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{42835B90-7B58-4D9C-99DA-22F82FBF39BF}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja2" sheetId="3" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Carga (kN)</t>
   </si>
@@ -29,6 +42,57 @@
   </si>
   <si>
     <t>Datos medidos</t>
+  </si>
+  <si>
+    <t>Parametros Viga</t>
+  </si>
+  <si>
+    <t>E (Gpa)</t>
+  </si>
+  <si>
+    <t>Luz entre los apoyos</t>
+  </si>
+  <si>
+    <t>Ancho</t>
+  </si>
+  <si>
+    <t>Altura</t>
+  </si>
+  <si>
+    <t>Módulo de elasticidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> P (Carga en kN)</t>
+  </si>
+  <si>
+    <t>δ (Deflexión en mm)</t>
+  </si>
+  <si>
+    <t>L (mm)</t>
+  </si>
+  <si>
+    <t>b(mm)</t>
+  </si>
+  <si>
+    <t>h (mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> I (Inercia Viga en mm^4)</t>
+  </si>
+  <si>
+    <t>Comparación</t>
+  </si>
+  <si>
+    <t>Deflexión teórica</t>
+  </si>
+  <si>
+    <t>Diferencia relativa</t>
+  </si>
+  <si>
+    <t>Defelexion teórica (mm)</t>
+  </si>
+  <si>
+    <t>Deflexión real(mm)</t>
   </si>
 </sst>
 </file>
@@ -352,7 +416,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -482,8 +546,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -526,13 +601,16 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="42" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Énfasis3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -568,6 +646,7 @@
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Notas" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Porcentaje" xfId="42" builtinId="5"/>
     <cellStyle name="Salida" xfId="10" builtinId="21" customBuiltin="1"/>
     <cellStyle name="Texto de advertencia" xfId="14" builtinId="11" customBuiltin="1"/>
     <cellStyle name="Texto explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
@@ -587,6 +666,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>261939</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>33337</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>381001</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>81598</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C50066DB-EA49-33C8-8560-D574A0E28153}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2543177" y="2566987"/>
+          <a:ext cx="1757362" cy="591186"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -906,98 +1034,361 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F479A5EE-3026-4AC6-9B52-937E645E3D9C}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="15.59765625" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" customWidth="1"/>
+    <col min="2" max="2" width="17.59765625" customWidth="1"/>
+    <col min="4" max="4" width="12.265625" customWidth="1"/>
+    <col min="9" max="9" width="20.6640625" customWidth="1"/>
+    <col min="10" max="10" width="16.46484375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1"/>
+      <c r="I1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+        <v>10</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="2">
+        <f>4*1000</f>
+        <v>4000</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" s="2">
         <v>0</v>
       </c>
       <c r="B3" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="D3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="2">
+        <f>0.2*1000</f>
+        <v>200</v>
+      </c>
+      <c r="F3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I3" s="2">
+        <f t="shared" ref="I3:I11" si="0">B15</f>
+        <v>0</v>
+      </c>
+      <c r="J3" s="2">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4">
+        <f>(J3-I3)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" s="2">
         <v>5</v>
       </c>
       <c r="B4" s="2">
         <v>0.26</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="D4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="2">
+        <f>0.4*1000</f>
+        <v>400</v>
+      </c>
+      <c r="F4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I4" s="2">
+        <f t="shared" si="0"/>
+        <v>0.25</v>
+      </c>
+      <c r="J4" s="2">
+        <v>0.26</v>
+      </c>
+      <c r="K4" s="4">
+        <f t="shared" ref="K4:K11" si="1">(J4-I4)/I4</f>
+        <v>4.0000000000000036E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" s="2">
         <v>10</v>
       </c>
       <c r="B5" s="2">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="D5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+      <c r="I5" s="2">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="J5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="K5" s="4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" s="2">
         <v>15</v>
       </c>
       <c r="B6" s="2">
         <v>0.76</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="I6" s="2">
+        <f t="shared" si="0"/>
+        <v>0.75</v>
+      </c>
+      <c r="J6" s="2">
+        <v>0.76</v>
+      </c>
+      <c r="K6" s="4">
+        <f t="shared" si="1"/>
+        <v>1.3333333333333345E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" s="2">
         <v>20</v>
       </c>
       <c r="B7" s="2">
         <v>1.01</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="D7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I7" s="2">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="J7" s="2">
+        <v>1.01</v>
+      </c>
+      <c r="K7" s="4">
+        <f t="shared" si="1"/>
+        <v>1.0000000000000009E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" s="2">
         <v>25</v>
       </c>
       <c r="B8" s="2">
         <v>1.28</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="D8">
+        <f>(E3*(E4^3))/12</f>
+        <v>1066666666.6666666</v>
+      </c>
+      <c r="I8" s="2">
+        <f t="shared" si="0"/>
+        <v>1.25</v>
+      </c>
+      <c r="J8" s="2">
+        <v>1.28</v>
+      </c>
+      <c r="K8" s="4">
+        <f t="shared" si="1"/>
+        <v>2.4000000000000021E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" s="2">
         <v>30</v>
       </c>
       <c r="B9" s="2">
         <v>1.54</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="I9" s="2">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
+      <c r="J9" s="2">
+        <v>1.54</v>
+      </c>
+      <c r="K9" s="4">
+        <f t="shared" si="1"/>
+        <v>2.6666666666666689E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" s="2">
         <v>35</v>
       </c>
       <c r="B10" s="2">
         <v>1.77</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="I10" s="2">
+        <f t="shared" si="0"/>
+        <v>1.75</v>
+      </c>
+      <c r="J10" s="2">
+        <v>1.77</v>
+      </c>
+      <c r="K10" s="4">
+        <f t="shared" si="1"/>
+        <v>1.1428571428571439E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" s="2">
         <v>40</v>
       </c>
       <c r="B11" s="2">
         <v>2.0499999999999998</v>
       </c>
+      <c r="I11" s="2">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="J11" s="2">
+        <v>2.0499999999999998</v>
+      </c>
+      <c r="K11" s="4">
+        <f t="shared" si="1"/>
+        <v>2.4999999999999911E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A13" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A14" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A15" s="2">
+        <v>0</v>
+      </c>
+      <c r="B15" s="2">
+        <f>(($E$2^3)*A15)/(48*$E$5*$D$8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A16" s="2">
+        <v>5</v>
+      </c>
+      <c r="B16" s="2">
+        <f t="shared" ref="B16:B23" si="2">(($E$2^3)*A16)/(48*$E$5*$D$8)</f>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A17" s="2">
+        <v>10</v>
+      </c>
+      <c r="B17" s="2">
+        <f t="shared" si="2"/>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A18" s="2">
+        <v>15</v>
+      </c>
+      <c r="B18" s="2">
+        <f t="shared" si="2"/>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A19" s="2">
+        <v>20</v>
+      </c>
+      <c r="B19" s="2">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A20" s="2">
+        <v>25</v>
+      </c>
+      <c r="B20" s="2">
+        <f t="shared" si="2"/>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A21" s="2">
+        <v>30</v>
+      </c>
+      <c r="B21" s="2">
+        <f t="shared" si="2"/>
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A22" s="2">
+        <v>35</v>
+      </c>
+      <c r="B22" s="2">
+        <f t="shared" si="2"/>
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A23" s="2">
+        <v>40</v>
+      </c>
+      <c r="B23" s="2">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A25" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
agrega verificación adicional y gráfico carga vs deflexión
</commit_message>
<xml_diff>
--- a/analysis/analisis_viga.xlsx
+++ b/analysis/analisis_viga.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\galej\Desktop\EVALUACION 1\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B16B76B5-5DF2-46A3-9E7B-9860B0FA41C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC0685F4-745C-48BA-B404-97528173C3D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{42835B90-7B58-4D9C-99DA-22F82FBF39BF}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja2" sheetId="3" r:id="rId1"/>
+    <sheet name="Calculos" sheetId="3" r:id="rId1"/>
+    <sheet name="Gráfico" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,8 +33,27 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={BED67B36-F9E6-4B9C-A5D2-56BA2AD5CBE9}</author>
+  </authors>
+  <commentList>
+    <comment ref="I13" authorId="0" shapeId="0" xr:uid="{BED67B36-F9E6-4B9C-A5D2-56BA2AD5CBE9}">
+      <text>
+        <t xml:space="preserve">[Comentario encadenado]
+Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+Comentario:
+ La razón deflexión/carga presenta un valor promedio de  0,051 mm/Kn, con un coef. de variación  de menos del 1%. Esta  constancia confirma que la viga opera dentro del régimen elástico lineal y valida la consistencia de los datos experimentales. 
+</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
   <si>
     <t>Carga (kN)</t>
   </si>
@@ -89,17 +109,36 @@
     <t>Diferencia relativa</t>
   </si>
   <si>
-    <t>Defelexion teórica (mm)</t>
+    <t>Deflexión real(mm)</t>
   </si>
   <si>
-    <t>Deflexión real(mm)</t>
+    <t>Deflexión teórica (mm)</t>
+  </si>
+  <si>
+    <t>Verificación</t>
+  </si>
+  <si>
+    <t>Promedio δ/P</t>
+  </si>
+  <si>
+    <t>δ/P (mm/kN)</t>
+  </si>
+  <si>
+    <t>Desviación estandar  δ/P</t>
+  </si>
+  <si>
+    <t>mm/kN</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="172" formatCode="0.000"/>
+    <numFmt numFmtId="175" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -233,6 +272,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -603,12 +648,14 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="42" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="175" fontId="0" fillId="0" borderId="10" xfId="42" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -668,6 +715,1196 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-CL" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:t>Comparación Carga vs. Deflexión </a:t>
+            </a:r>
+            <a:endParaRPr lang="es-CL"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-CL"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Deflexión teórica</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Gráfico!$A$2:$A$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>40</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Gráfico!$B$2:$B$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.25</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.75</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.25</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.75</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-1442-4A97-B488-C68F6453AAE6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Deflexión real</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Gráfico!$A$2:$A$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>40</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Gráfico!$C$2:$C$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.26</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.76</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.01</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.28</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.54</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.77</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.0499999999999998</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-1442-4A97-B488-C68F6453AAE6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1929358224"/>
+        <c:axId val="2003646800"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1929358224"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="es-CL"/>
+                  <a:t>Carga</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="es-CL" baseline="0"/>
+                  <a:t> P (kN)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="es-CL"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2003646800"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="2003646800"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t> Deflexión </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="el-GR"/>
+                  <a:t>δ (</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>mm)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="es-CL"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CL"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1929358224"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-CL"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-CL"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
@@ -715,6 +1952,53 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>128587</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>161924</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>695324</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>9524</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Gráfico 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A2A797B0-963C-F6E3-3AC5-3362DD344E2E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Gabriela  Soto" id="{7F00B2C2-3996-4058-B6AE-7ED535477C25}" userId="S::gabriela.soto.g@usach.cl::e57b149e-2ef5-4ecc-88a0-4c04e6363b38" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1032,9 +2316,19 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="I13" dT="2026-10-05T14:16:32.12" personId="{7F00B2C2-3996-4058-B6AE-7ED535477C25}" id="{BED67B36-F9E6-4B9C-A5D2-56BA2AD5CBE9}">
+    <text xml:space="preserve">
+ La razón deflexión/carga presenta un valor promedio de  0,051 mm/Kn, con un coef. de variación  de menos del 1%. Esta  constancia confirma que la viga opera dentro del régimen elástico lineal y valida la consistencia de los datos experimentales. 
+</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F479A5EE-3026-4AC6-9B52-937E645E3D9C}">
-  <dimension ref="A1:K25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F479A5EE-3026-4AC6-9B52-937E645E3D9C}">
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14.33203125" customWidth="1"/>
@@ -1042,6 +2336,7 @@
     <col min="4" max="4" width="12.265625" customWidth="1"/>
     <col min="9" max="9" width="20.6640625" customWidth="1"/>
     <col min="10" max="10" width="16.46484375" customWidth="1"/>
+    <col min="12" max="12" width="12.53125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.45">
@@ -1074,10 +2369,10 @@
         <v>5</v>
       </c>
       <c r="I2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" t="s">
         <v>18</v>
-      </c>
-      <c r="J2" t="s">
-        <v>19</v>
       </c>
       <c r="K2" t="s">
         <v>17</v>
@@ -1294,6 +2589,9 @@
       <c r="A13" s="1" t="s">
         <v>16</v>
       </c>
+      <c r="I13" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
@@ -1302,6 +2600,17 @@
       <c r="B14" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="I14" s="2" t="str">
+        <f t="shared" ref="I14:I23" si="2">A2</f>
+        <v xml:space="preserve"> P (Carga en kN)</v>
+      </c>
+      <c r="J14" s="2" t="str">
+        <f t="shared" ref="J14:J23" si="3">B2</f>
+        <v>δ (Deflexión en mm)</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A15" s="2">
@@ -1311,81 +2620,354 @@
         <f>(($E$2^3)*A15)/(48*$E$5*$D$8)</f>
         <v>0</v>
       </c>
+      <c r="I15" s="2">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J15" s="2">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="K15" s="2"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A16" s="2">
         <v>5</v>
       </c>
       <c r="B16" s="2">
-        <f t="shared" ref="B16:B23" si="2">(($E$2^3)*A16)/(48*$E$5*$D$8)</f>
+        <f t="shared" ref="B16:B23" si="4">(($E$2^3)*A16)/(48*$E$5*$D$8)</f>
         <v>0.25</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="I16" s="2">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="J16" s="2">
+        <f t="shared" si="3"/>
+        <v>0.26</v>
+      </c>
+      <c r="K16" s="2">
+        <f>J16/I16</f>
+        <v>5.2000000000000005E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A17" s="2">
         <v>10</v>
       </c>
       <c r="B17" s="2">
+        <f t="shared" si="4"/>
+        <v>0.5</v>
+      </c>
+      <c r="I17" s="2">
         <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="J17" s="2">
+        <f t="shared" si="3"/>
         <v>0.5</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="K17" s="2">
+        <f t="shared" ref="K17:K23" si="5">J17/I17</f>
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A18" s="2">
         <v>15</v>
       </c>
       <c r="B18" s="2">
+        <f t="shared" si="4"/>
+        <v>0.75</v>
+      </c>
+      <c r="I18" s="2">
         <f t="shared" si="2"/>
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+        <v>15</v>
+      </c>
+      <c r="J18" s="2">
+        <f t="shared" si="3"/>
+        <v>0.76</v>
+      </c>
+      <c r="K18" s="2">
+        <f t="shared" si="5"/>
+        <v>5.0666666666666665E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A19" s="2">
         <v>20</v>
       </c>
       <c r="B19" s="2">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="I19" s="2">
         <f t="shared" si="2"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+        <v>20</v>
+      </c>
+      <c r="J19" s="2">
+        <f t="shared" si="3"/>
+        <v>1.01</v>
+      </c>
+      <c r="K19" s="2">
+        <f t="shared" si="5"/>
+        <v>5.0500000000000003E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A20" s="2">
         <v>25</v>
       </c>
       <c r="B20" s="2">
+        <f t="shared" si="4"/>
+        <v>1.25</v>
+      </c>
+      <c r="I20" s="2">
         <f t="shared" si="2"/>
-        <v>1.25</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+        <v>25</v>
+      </c>
+      <c r="J20" s="2">
+        <f t="shared" si="3"/>
+        <v>1.28</v>
+      </c>
+      <c r="K20" s="2">
+        <f t="shared" si="5"/>
+        <v>5.1200000000000002E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A21" s="2">
         <v>30</v>
       </c>
       <c r="B21" s="2">
+        <f t="shared" si="4"/>
+        <v>1.5</v>
+      </c>
+      <c r="I21" s="2">
         <f t="shared" si="2"/>
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+        <v>30</v>
+      </c>
+      <c r="J21" s="2">
+        <f t="shared" si="3"/>
+        <v>1.54</v>
+      </c>
+      <c r="K21" s="2">
+        <f t="shared" si="5"/>
+        <v>5.1333333333333335E-2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A22" s="2">
         <v>35</v>
       </c>
       <c r="B22" s="2">
+        <f t="shared" si="4"/>
+        <v>1.75</v>
+      </c>
+      <c r="I22" s="2">
         <f t="shared" si="2"/>
-        <v>1.75</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+        <v>35</v>
+      </c>
+      <c r="J22" s="2">
+        <f t="shared" si="3"/>
+        <v>1.77</v>
+      </c>
+      <c r="K22" s="2">
+        <f t="shared" si="5"/>
+        <v>5.0571428571428573E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A23" s="2">
         <v>40</v>
       </c>
       <c r="B23" s="2">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="I23" s="2">
         <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="J23" s="2">
+        <f t="shared" si="3"/>
+        <v>2.0499999999999998</v>
+      </c>
+      <c r="K23" s="2">
+        <f t="shared" si="5"/>
+        <v>5.1249999999999997E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A25" s="1"/>
+      <c r="I25" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J25" s="5">
+        <f>AVERAGE(K16:K23)</f>
+        <v>5.0940178571428574E-2</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="I26" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J26" s="6">
+        <f>_xlfn.STDEV.S(K16:K23)</f>
+        <v>6.2447313393879339E-4</v>
+      </c>
+      <c r="K26" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A68BF21B-EC22-431C-80C5-6E31AC1DC882}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="16.265625" customWidth="1"/>
+    <col min="2" max="2" width="20.73046875" customWidth="1"/>
+    <col min="3" max="3" width="19.06640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="2" t="str">
+        <f>Calculos!I2</f>
+        <v>Deflexión teórica (mm)</v>
+      </c>
+      <c r="C1" s="2" t="str">
+        <f>Calculos!J2</f>
+        <v>Deflexión real(mm)</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" s="2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2">
+        <f>Calculos!I3</f>
+        <v>0</v>
+      </c>
+      <c r="C2" s="2">
+        <f>Calculos!J3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" s="2">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2">
+        <f>Calculos!I4</f>
+        <v>0.25</v>
+      </c>
+      <c r="C3" s="2">
+        <f>Calculos!J4</f>
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" s="2">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2">
+        <f>Calculos!I5</f>
+        <v>0.5</v>
+      </c>
+      <c r="C4" s="2">
+        <f>Calculos!J5</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" s="2">
+        <v>15</v>
+      </c>
+      <c r="B5" s="2">
+        <f>Calculos!I6</f>
+        <v>0.75</v>
+      </c>
+      <c r="C5" s="2">
+        <f>Calculos!J6</f>
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" s="2">
+        <v>20</v>
+      </c>
+      <c r="B6" s="2">
+        <f>Calculos!I7</f>
+        <v>1</v>
+      </c>
+      <c r="C6" s="2">
+        <f>Calculos!J7</f>
+        <v>1.01</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" s="2">
+        <v>25</v>
+      </c>
+      <c r="B7" s="2">
+        <f>Calculos!I8</f>
+        <v>1.25</v>
+      </c>
+      <c r="C7" s="2">
+        <f>Calculos!J8</f>
+        <v>1.28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" s="2">
+        <v>30</v>
+      </c>
+      <c r="B8" s="2">
+        <f>Calculos!I9</f>
+        <v>1.5</v>
+      </c>
+      <c r="C8" s="2">
+        <f>Calculos!J9</f>
+        <v>1.54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" s="2">
+        <v>35</v>
+      </c>
+      <c r="B9" s="2">
+        <f>Calculos!I10</f>
+        <v>1.75</v>
+      </c>
+      <c r="C9" s="2">
+        <f>Calculos!J10</f>
+        <v>1.77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" s="2">
+        <v>40</v>
+      </c>
+      <c r="B10" s="2">
+        <f>Calculos!I11</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A25" s="1"/>
+      <c r="C10" s="2">
+        <f>Calculos!J11</f>
+        <v>2.0499999999999998</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
se corrigen datos de verificación
</commit_message>
<xml_diff>
--- a/analysis/analisis_viga.xlsx
+++ b/analysis/analisis_viga.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\galej\Desktop\EVALUACION 1\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC0685F4-745C-48BA-B404-97528173C3D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49BB253C-DD60-453F-ADA1-5500336A6471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{42835B90-7B58-4D9C-99DA-22F82FBF39BF}"/>
   </bookViews>
@@ -44,7 +44,7 @@
         <t xml:space="preserve">[Comentario encadenado]
 Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
 Comentario:
- La razón deflexión/carga presenta un valor promedio de  0,051 mm/Kn, con un coef. de variación  de menos del 1%. Esta  constancia confirma que la viga opera dentro del régimen elástico lineal y valida la consistencia de los datos experimentales. 
+ La razón deflexión/carga presenta un valor promedio de  0,051 mm/Kn, con un coef. de variación  de menos del 2%. Esta  constancia confirma que la viga opera dentro del régimen elástico lineal y valida la consistencia de los datos experimentales. 
 </t>
       </text>
     </comment>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
   <si>
     <t>Carga (kN)</t>
   </si>
@@ -129,16 +129,19 @@
   <si>
     <t>mm/kN</t>
   </si>
+  <si>
+    <t>Coef. De Variación</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="172" formatCode="0.000"/>
-    <numFmt numFmtId="175" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="171" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -272,12 +275,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -648,14 +645,15 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="42" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="175" fontId="0" fillId="0" borderId="10" xfId="42" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="10" xfId="42" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="10" xfId="42" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2320,7 +2318,7 @@
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="I13" dT="2026-10-05T14:16:32.12" personId="{7F00B2C2-3996-4058-B6AE-7ED535477C25}" id="{BED67B36-F9E6-4B9C-A5D2-56BA2AD5CBE9}">
     <text xml:space="preserve">
- La razón deflexión/carga presenta un valor promedio de  0,051 mm/Kn, con un coef. de variación  de menos del 1%. Esta  constancia confirma que la viga opera dentro del régimen elástico lineal y valida la consistencia de los datos experimentales. 
+ La razón deflexión/carga presenta un valor promedio de  0,051 mm/Kn, con un coef. de variación  de menos del 2%. Esta  constancia confirma que la viga opera dentro del régimen elástico lineal y valida la consistencia de los datos experimentales. 
 </text>
   </threadedComment>
 </ThreadedComments>
@@ -2328,7 +2326,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F479A5EE-3026-4AC6-9B52-937E645E3D9C}">
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14.33203125" customWidth="1"/>
@@ -2819,7 +2817,18 @@
         <f>_xlfn.STDEV.S(K16:K23)</f>
         <v>6.2447313393879339E-4</v>
       </c>
-      <c r="K26" s="2"/>
+      <c r="K26" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="I27" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J27" s="7">
+        <f>J26/J25</f>
+        <v>1.2258950625058255E-2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>